<commit_message>
commit Sport Data muestra .xlsx
</commit_message>
<xml_diff>
--- a/estadistica-excel/SportData_muestra.xlsx
+++ b/estadistica-excel/SportData_muestra.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Proyectos/cursos_activos/inserta_once/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UsuarioM\Documents\curso_big_data_paula\ejercicio_rombo_y_estadistica_excel\estadistica-excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EBA25B7-521E-EB4F-B673-F588AB60EF5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9487136C-C550-4D0B-A056-93024BAECAC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37300" yWindow="1080" windowWidth="36000" windowHeight="19740" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="29952" windowHeight="15708" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Datos!$A$1:$N$201</definedName>
@@ -35,8 +36,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1214" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1216" uniqueCount="49">
   <si>
     <t>ID_Venta</t>
   </si>
@@ -181,14 +204,16 @@
   <si>
     <t>Botella térmica</t>
   </si>
+  <si>
+    <t>FILTRO</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-    <numFmt numFmtId="165" formatCode="#,##0.00\ _€"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#,##0.00\ _€"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -269,21 +294,21 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -554,7 +579,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N201"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
@@ -571,7 +596,7 @@
     <col min="14" max="14" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="26.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" ht="26.7" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -615,7 +640,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>1001</v>
       </c>
@@ -661,7 +686,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>1002</v>
       </c>
@@ -707,7 +732,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>1003</v>
       </c>
@@ -753,7 +778,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>1004</v>
       </c>
@@ -799,7 +824,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <v>1005</v>
       </c>
@@ -845,7 +870,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5">
         <v>1006</v>
       </c>
@@ -891,7 +916,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <v>1007</v>
       </c>
@@ -937,7 +962,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
         <v>1008</v>
       </c>
@@ -983,7 +1008,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2">
         <v>1009</v>
       </c>
@@ -1029,7 +1054,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2">
         <v>1010</v>
       </c>
@@ -1075,7 +1100,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5">
         <v>1011</v>
       </c>
@@ -1121,7 +1146,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="13" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5">
         <v>1012</v>
       </c>
@@ -1167,7 +1192,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5">
         <v>1013</v>
       </c>
@@ -1213,7 +1238,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="5">
         <v>1014</v>
       </c>
@@ -1259,7 +1284,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2">
         <v>1015</v>
       </c>
@@ -1305,7 +1330,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>1016</v>
       </c>
@@ -1351,7 +1376,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5">
         <v>1017</v>
       </c>
@@ -1397,7 +1422,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>1018</v>
       </c>
@@ -1443,7 +1468,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5">
         <v>1019</v>
       </c>
@@ -1489,7 +1514,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>1020</v>
       </c>
@@ -1535,7 +1560,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>1021</v>
       </c>
@@ -1581,7 +1606,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="5">
         <v>1022</v>
       </c>
@@ -1627,7 +1652,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5">
         <v>1023</v>
       </c>
@@ -1673,7 +1698,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="5">
         <v>1024</v>
       </c>
@@ -1719,7 +1744,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>1025</v>
       </c>
@@ -1765,7 +1790,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>1026</v>
       </c>
@@ -1811,7 +1836,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>1027</v>
       </c>
@@ -1857,7 +1882,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>1028</v>
       </c>
@@ -1903,7 +1928,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>1029</v>
       </c>
@@ -1949,7 +1974,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>1030</v>
       </c>
@@ -1995,7 +2020,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>1031</v>
       </c>
@@ -2041,7 +2066,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="2">
         <v>1032</v>
       </c>
@@ -2087,7 +2112,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="5">
         <v>1033</v>
       </c>
@@ -2133,7 +2158,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="5">
         <v>1034</v>
       </c>
@@ -2179,7 +2204,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5">
         <v>1035</v>
       </c>
@@ -2225,7 +2250,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="5">
         <v>1036</v>
       </c>
@@ -2271,7 +2296,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="38" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5">
         <v>1037</v>
       </c>
@@ -2317,7 +2342,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="39" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="2">
         <v>1038</v>
       </c>
@@ -2363,7 +2388,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="5">
         <v>1039</v>
       </c>
@@ -2409,7 +2434,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="41" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="2">
         <v>1040</v>
       </c>
@@ -2455,7 +2480,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="42" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5">
         <v>1041</v>
       </c>
@@ -2501,7 +2526,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="43" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="2">
         <v>1042</v>
       </c>
@@ -2547,7 +2572,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="44" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5">
         <v>1043</v>
       </c>
@@ -2593,7 +2618,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="45" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="2">
         <v>1044</v>
       </c>
@@ -2639,7 +2664,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="46" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="5">
         <v>1045</v>
       </c>
@@ -2685,7 +2710,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="2">
         <v>1046</v>
       </c>
@@ -2731,7 +2756,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="48" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="2">
         <v>1047</v>
       </c>
@@ -2777,7 +2802,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="49" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="2">
         <v>1048</v>
       </c>
@@ -2823,7 +2848,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="50" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="2">
         <v>1049</v>
       </c>
@@ -2869,7 +2894,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="51" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="2">
         <v>1050</v>
       </c>
@@ -2915,7 +2940,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="52" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="5">
         <v>1051</v>
       </c>
@@ -2961,7 +2986,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="53" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="2">
         <v>1052</v>
       </c>
@@ -3007,7 +3032,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="54" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="2">
         <v>1053</v>
       </c>
@@ -3053,7 +3078,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="55" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="5">
         <v>1054</v>
       </c>
@@ -3099,7 +3124,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="56" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="2">
         <v>1055</v>
       </c>
@@ -3145,7 +3170,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="57" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="5">
         <v>1056</v>
       </c>
@@ -3191,7 +3216,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="58" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="5">
         <v>1057</v>
       </c>
@@ -3237,7 +3262,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="59" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="5">
         <v>1058</v>
       </c>
@@ -3283,7 +3308,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="60" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="2">
         <v>1059</v>
       </c>
@@ -3329,7 +3354,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="61" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="2">
         <v>1060</v>
       </c>
@@ -3375,7 +3400,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="5">
         <v>1061</v>
       </c>
@@ -3421,7 +3446,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="5">
         <v>1062</v>
       </c>
@@ -3467,7 +3492,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="64" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="2">
         <v>1063</v>
       </c>
@@ -3513,7 +3538,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="65" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A65" s="2">
         <v>1064</v>
       </c>
@@ -3559,7 +3584,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="66" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="5">
         <v>1065</v>
       </c>
@@ -3605,7 +3630,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="67" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="2">
         <v>1066</v>
       </c>
@@ -3651,7 +3676,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="68" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="5">
         <v>1067</v>
       </c>
@@ -3697,7 +3722,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="69" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A69" s="5">
         <v>1068</v>
       </c>
@@ -3743,7 +3768,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="70" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" s="5">
         <v>1069</v>
       </c>
@@ -3789,7 +3814,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="71" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5">
         <v>1070</v>
       </c>
@@ -3835,7 +3860,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="72" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="5">
         <v>1071</v>
       </c>
@@ -3881,7 +3906,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="73" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A73" s="2">
         <v>1072</v>
       </c>
@@ -3927,7 +3952,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="74" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="5">
         <v>1073</v>
       </c>
@@ -3973,7 +3998,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="75" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="5">
         <v>1074</v>
       </c>
@@ -4019,7 +4044,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="76" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="2">
         <v>1075</v>
       </c>
@@ -4065,7 +4090,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="77" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A77" s="5">
         <v>1076</v>
       </c>
@@ -4111,7 +4136,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="78" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" s="5">
         <v>1077</v>
       </c>
@@ -4157,7 +4182,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="79" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="2">
         <v>1078</v>
       </c>
@@ -4203,7 +4228,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="80" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="2">
         <v>1079</v>
       </c>
@@ -4249,7 +4274,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="81" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="5">
         <v>1080</v>
       </c>
@@ -4295,7 +4320,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="82" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="5">
         <v>1081</v>
       </c>
@@ -4341,7 +4366,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="83" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="2">
         <v>1082</v>
       </c>
@@ -4387,7 +4412,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="84" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A84" s="2">
         <v>1083</v>
       </c>
@@ -4433,7 +4458,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="85" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A85" s="2">
         <v>1084</v>
       </c>
@@ -4479,7 +4504,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="86" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" s="2">
         <v>1085</v>
       </c>
@@ -4525,7 +4550,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="87" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A87" s="5">
         <v>1086</v>
       </c>
@@ -4571,7 +4596,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="88" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A88" s="5">
         <v>1087</v>
       </c>
@@ -4617,7 +4642,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="89" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A89" s="5">
         <v>1088</v>
       </c>
@@ -4663,7 +4688,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="90" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" s="5">
         <v>1089</v>
       </c>
@@ -4709,7 +4734,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="91" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A91" s="2">
         <v>1090</v>
       </c>
@@ -4755,7 +4780,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="92" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="2">
         <v>1091</v>
       </c>
@@ -4801,7 +4826,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="93" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="2">
         <v>1092</v>
       </c>
@@ -4847,7 +4872,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="94" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" s="2">
         <v>1093</v>
       </c>
@@ -4893,7 +4918,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="95" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="5">
         <v>1094</v>
       </c>
@@ -4939,7 +4964,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="96" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="2">
         <v>1095</v>
       </c>
@@ -4985,7 +5010,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="97" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A97" s="2">
         <v>1096</v>
       </c>
@@ -5031,7 +5056,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="98" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" s="5">
         <v>1097</v>
       </c>
@@ -5077,7 +5102,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="99" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A99" s="2">
         <v>1098</v>
       </c>
@@ -5123,7 +5148,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="100" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A100" s="2">
         <v>1099</v>
       </c>
@@ -5169,7 +5194,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="101" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="5">
         <v>1100</v>
       </c>
@@ -5215,7 +5240,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="102" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="5">
         <v>1101</v>
       </c>
@@ -5261,7 +5286,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="103" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="2">
         <v>1102</v>
       </c>
@@ -5307,7 +5332,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="104" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="5">
         <v>1103</v>
       </c>
@@ -5353,7 +5378,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="105" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="5">
         <v>1104</v>
       </c>
@@ -5399,7 +5424,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="106" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="2">
         <v>1105</v>
       </c>
@@ -5445,7 +5470,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="107" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="2">
         <v>1106</v>
       </c>
@@ -5491,7 +5516,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="108" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A108" s="5">
         <v>1107</v>
       </c>
@@ -5537,7 +5562,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="109" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A109" s="5">
         <v>1108</v>
       </c>
@@ -5583,7 +5608,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="110" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" s="2">
         <v>1109</v>
       </c>
@@ -5629,7 +5654,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="111" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A111" s="5">
         <v>1110</v>
       </c>
@@ -5675,7 +5700,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="112" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="2">
         <v>1111</v>
       </c>
@@ -5721,7 +5746,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="113" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A113" s="5">
         <v>1112</v>
       </c>
@@ -5767,7 +5792,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="114" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="2">
         <v>1113</v>
       </c>
@@ -5813,7 +5838,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="115" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A115" s="2">
         <v>1114</v>
       </c>
@@ -5859,7 +5884,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="116" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A116" s="5">
         <v>1115</v>
       </c>
@@ -5905,7 +5930,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="117" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A117" s="5">
         <v>1116</v>
       </c>
@@ -5951,7 +5976,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="118" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" s="2">
         <v>1117</v>
       </c>
@@ -5997,7 +6022,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="119" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="5">
         <v>1118</v>
       </c>
@@ -6043,7 +6068,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="120" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="2">
         <v>1119</v>
       </c>
@@ -6089,7 +6114,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="121" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A121" s="5">
         <v>1120</v>
       </c>
@@ -6135,7 +6160,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="122" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" s="2">
         <v>1121</v>
       </c>
@@ -6181,7 +6206,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="123" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="5">
         <v>1122</v>
       </c>
@@ -6227,7 +6252,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="124" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="5">
         <v>1123</v>
       </c>
@@ -6273,7 +6298,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="125" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A125" s="2">
         <v>1124</v>
       </c>
@@ -6319,7 +6344,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="126" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" s="5">
         <v>1125</v>
       </c>
@@ -6365,7 +6390,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="127" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A127" s="5">
         <v>1126</v>
       </c>
@@ -6411,7 +6436,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="128" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A128" s="2">
         <v>1127</v>
       </c>
@@ -6457,7 +6482,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="129" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A129" s="5">
         <v>1128</v>
       </c>
@@ -6503,7 +6528,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="130" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="2">
         <v>1129</v>
       </c>
@@ -6549,7 +6574,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="131" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="2">
         <v>1130</v>
       </c>
@@ -6595,7 +6620,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="132" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="2">
         <v>1131</v>
       </c>
@@ -6641,7 +6666,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="133" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A133" s="2">
         <v>1132</v>
       </c>
@@ -6687,7 +6712,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="134" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" s="2">
         <v>1133</v>
       </c>
@@ -6733,7 +6758,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="135" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A135" s="5">
         <v>1134</v>
       </c>
@@ -6779,7 +6804,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="136" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A136" s="5">
         <v>1135</v>
       </c>
@@ -6825,7 +6850,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="137" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A137" s="5">
         <v>1136</v>
       </c>
@@ -6871,7 +6896,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="138" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="5">
         <v>1137</v>
       </c>
@@ -6917,7 +6942,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="139" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A139" s="2">
         <v>1138</v>
       </c>
@@ -6963,7 +6988,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="140" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" s="2">
         <v>1139</v>
       </c>
@@ -7009,7 +7034,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="141" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A141" s="2">
         <v>1140</v>
       </c>
@@ -7055,7 +7080,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="142" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" s="5">
         <v>1141</v>
       </c>
@@ -7101,7 +7126,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="143" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A143" s="2">
         <v>1142</v>
       </c>
@@ -7147,7 +7172,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="144" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A144" s="2">
         <v>1143</v>
       </c>
@@ -7193,7 +7218,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="145" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A145" s="2">
         <v>1144</v>
       </c>
@@ -7239,7 +7264,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="146" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" s="2">
         <v>1145</v>
       </c>
@@ -7285,7 +7310,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="147" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A147" s="5">
         <v>1146</v>
       </c>
@@ -7331,7 +7356,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="148" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A148" s="2">
         <v>1147</v>
       </c>
@@ -7377,7 +7402,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="149" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A149" s="2">
         <v>1148</v>
       </c>
@@ -7423,7 +7448,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="150" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" s="5">
         <v>1149</v>
       </c>
@@ -7469,7 +7494,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="151" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A151" s="2">
         <v>1150</v>
       </c>
@@ -7515,7 +7540,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="152" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A152" s="5">
         <v>1151</v>
       </c>
@@ -7561,7 +7586,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="153" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A153" s="5">
         <v>1152</v>
       </c>
@@ -7607,7 +7632,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="154" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" s="5">
         <v>1153</v>
       </c>
@@ -7653,7 +7678,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="155" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A155" s="5">
         <v>1154</v>
       </c>
@@ -7699,7 +7724,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="156" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A156" s="5">
         <v>1155</v>
       </c>
@@ -7745,7 +7770,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="157" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A157" s="2">
         <v>1156</v>
       </c>
@@ -7791,7 +7816,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="158" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" s="5">
         <v>1157</v>
       </c>
@@ -7837,7 +7862,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="159" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A159" s="5">
         <v>1158</v>
       </c>
@@ -7883,7 +7908,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="160" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A160" s="2">
         <v>1159</v>
       </c>
@@ -7929,7 +7954,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="161" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A161" s="5">
         <v>1160</v>
       </c>
@@ -7975,7 +8000,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="162" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A162" s="5">
         <v>1161</v>
       </c>
@@ -8021,7 +8046,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="163" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A163" s="2">
         <v>1162</v>
       </c>
@@ -8067,7 +8092,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="164" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A164" s="2">
         <v>1163</v>
       </c>
@@ -8113,7 +8138,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="165" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A165" s="5">
         <v>1164</v>
       </c>
@@ -8159,7 +8184,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="166" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A166" s="2">
         <v>1165</v>
       </c>
@@ -8205,7 +8230,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="167" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A167" s="5">
         <v>1166</v>
       </c>
@@ -8251,7 +8276,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="168" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A168" s="5">
         <v>1167</v>
       </c>
@@ -8297,7 +8322,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="169" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A169" s="2">
         <v>1168</v>
       </c>
@@ -8343,7 +8368,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="170" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A170" s="2">
         <v>1169</v>
       </c>
@@ -8389,7 +8414,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="171" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A171" s="2">
         <v>1170</v>
       </c>
@@ -8435,7 +8460,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="172" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A172" s="2">
         <v>1171</v>
       </c>
@@ -8481,7 +8506,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="173" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A173" s="2">
         <v>1172</v>
       </c>
@@ -8527,7 +8552,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="174" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A174" s="2">
         <v>1173</v>
       </c>
@@ -8573,7 +8598,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="175" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A175" s="2">
         <v>1174</v>
       </c>
@@ -8619,7 +8644,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="176" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A176" s="2">
         <v>1175</v>
       </c>
@@ -8665,7 +8690,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="177" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A177" s="5">
         <v>1176</v>
       </c>
@@ -8711,7 +8736,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="178" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A178" s="5">
         <v>1177</v>
       </c>
@@ -8757,7 +8782,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="179" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A179" s="5">
         <v>1178</v>
       </c>
@@ -8803,7 +8828,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="180" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A180" s="5">
         <v>1179</v>
       </c>
@@ -8849,7 +8874,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="181" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A181" s="5">
         <v>1180</v>
       </c>
@@ -8895,7 +8920,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="182" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A182" s="5">
         <v>1181</v>
       </c>
@@ -8941,7 +8966,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="183" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A183" s="5">
         <v>1182</v>
       </c>
@@ -8987,7 +9012,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="184" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A184" s="5">
         <v>1183</v>
       </c>
@@ -9033,7 +9058,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="185" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A185" s="2">
         <v>1184</v>
       </c>
@@ -9079,7 +9104,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="186" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A186" s="5">
         <v>1185</v>
       </c>
@@ -9125,7 +9150,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="187" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A187" s="5">
         <v>1186</v>
       </c>
@@ -9171,7 +9196,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="188" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A188" s="5">
         <v>1187</v>
       </c>
@@ -9217,7 +9242,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="189" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A189" s="2">
         <v>1188</v>
       </c>
@@ -9263,7 +9288,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="190" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A190" s="5">
         <v>1189</v>
       </c>
@@ -9309,7 +9334,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="191" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A191" s="5">
         <v>1190</v>
       </c>
@@ -9355,7 +9380,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="192" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A192" s="2">
         <v>1191</v>
       </c>
@@ -9401,7 +9426,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="193" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A193" s="5">
         <v>1192</v>
       </c>
@@ -9447,7 +9472,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="194" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A194" s="5">
         <v>1193</v>
       </c>
@@ -9483,7 +9508,7 @@
         <v>5.17</v>
       </c>
       <c r="L194" s="10">
-        <f t="shared" ref="L194:L225" si="13">J194-K194</f>
+        <f t="shared" ref="L194:L201" si="13">J194-K194</f>
         <v>12.08</v>
       </c>
       <c r="M194" s="5" t="s">
@@ -9493,7 +9518,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="195" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A195" s="5">
         <v>1194</v>
       </c>
@@ -9539,7 +9564,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="196" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A196" s="2">
         <v>1195</v>
       </c>
@@ -9585,7 +9610,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="197" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A197" s="2">
         <v>1196</v>
       </c>
@@ -9631,7 +9656,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="198" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A198" s="2">
         <v>1197</v>
       </c>
@@ -9677,7 +9702,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="199" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A199" s="5">
         <v>1198</v>
       </c>
@@ -9723,7 +9748,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="200" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A200" s="5">
         <v>1199</v>
       </c>
@@ -9769,7 +9794,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="201" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A201" s="2">
         <v>1200</v>
       </c>
@@ -9821,7 +9846,48 @@
       <sortCondition ref="A1:A201"/>
     </sortState>
   </autoFilter>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1:D1048576" xr:uid="{81B4F683-5A99-46EB-8901-F560BEB881F5}">
+      <formula1>$D:$D</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{02238965-6401-4845-908C-F46DC5B4E1B8}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="e" cm="1">
+        <f t="array" ref="A2">_xlfn._xlws.FILTER(Datos!A1:N201,Datos!D:D=B1)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{342E0E64-DE4C-40BD-928D-ADD56E663E4B}">
+          <x14:formula1>
+            <xm:f>Datos!$D:$D</xm:f>
+          </x14:formula1>
+          <xm:sqref>B1</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
 </file>
</xml_diff>